<commit_message>
feat: select commit and branch
</commit_message>
<xml_diff>
--- a/database/data_dictionary.xlsx
+++ b/database/data_dictionary.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Duck\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Duck\Desktop\Taller\veraud\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5012FCE-50D0-4AA8-9DCA-1BBA2C576A53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C64DC17-9BA1-407A-B009-C23754C8BFBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{C4133E00-A44A-4AC3-8FAA-A9370F47246C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="67">
   <si>
     <t>PK</t>
   </si>
@@ -219,6 +219,24 @@
   </si>
   <si>
     <t>General note: UNIQUE (project_id, commit_hash)</t>
+  </si>
+  <si>
+    <t>task</t>
+  </si>
+  <si>
+    <t>kind</t>
+  </si>
+  <si>
+    <t>exit_code</t>
+  </si>
+  <si>
+    <t>log_trail</t>
+  </si>
+  <si>
+    <t>Values: defined by the application</t>
+  </si>
+  <si>
+    <t>Values: "Queued", "Running", "Failed"</t>
   </si>
 </sst>
 </file>
@@ -368,7 +386,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -465,6 +483,24 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -800,7 +836,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{790AE83E-F20F-4249-A016-8E165DBEC677}">
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" style="8" customWidth="1"/>
@@ -1635,6 +1671,108 @@
       <c r="F55" s="24"/>
       <c r="G55" s="24"/>
       <c r="H55" s="25"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A56" s="33" t="s">
+        <v>61</v>
+      </c>
+      <c r="B56" s="34" t="s">
+        <v>5</v>
+      </c>
+      <c r="C56" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="D56" s="35" t="s">
+        <v>37</v>
+      </c>
+      <c r="E56" s="35"/>
+      <c r="F56" s="35" t="s">
+        <v>7</v>
+      </c>
+      <c r="G56" s="35"/>
+      <c r="H56" s="36"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A57" s="7"/>
+      <c r="B57" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="C57" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="D57" s="38"/>
+      <c r="E57" s="38" t="s">
+        <v>37</v>
+      </c>
+      <c r="F57" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="G57" s="38"/>
+      <c r="H57" s="10"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A58" s="7"/>
+      <c r="B58" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="C58" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="D58" s="38"/>
+      <c r="E58" s="38"/>
+      <c r="F58" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="G58" s="38"/>
+      <c r="H58" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A59" s="7"/>
+      <c r="B59" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="C59" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="D59" s="38"/>
+      <c r="E59" s="38"/>
+      <c r="F59" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="G59" s="38"/>
+      <c r="H59" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A60" s="7"/>
+      <c r="B60" s="37" t="s">
+        <v>63</v>
+      </c>
+      <c r="C60" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="D60" s="38"/>
+      <c r="E60" s="38"/>
+      <c r="F60" s="38"/>
+      <c r="G60" s="38"/>
+      <c r="H60" s="10"/>
+    </row>
+    <row r="61" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A61" s="16"/>
+      <c r="B61" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="C61" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="D61" s="14"/>
+      <c r="E61" s="14"/>
+      <c r="F61" s="14"/>
+      <c r="G61" s="14"/>
+      <c r="H61" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>

<commit_message>
fix(db): change agent_execution state values
</commit_message>
<xml_diff>
--- a/database/data_dictionary.xlsx
+++ b/database/data_dictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Duck\Desktop\Taller\veraud\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C64DC17-9BA1-407A-B009-C23754C8BFBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8BBD8D1-9063-44C9-B9B6-F60DC68F3822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{C4133E00-A44A-4AC3-8FAA-A9370F47246C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="68">
   <si>
     <t>PK</t>
   </si>
@@ -237,6 +237,9 @@
   </si>
   <si>
     <t>Values: "Queued", "Running", "Failed"</t>
+  </si>
+  <si>
+    <t>result</t>
   </si>
 </sst>
 </file>
@@ -386,7 +389,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -454,6 +457,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -483,24 +498,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -836,7 +833,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{790AE83E-F20F-4249-A016-8E165DBEC677}">
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" style="8" customWidth="1"/>
@@ -848,16 +845,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
       <c r="I1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1026,14 +1023,14 @@
       <c r="H11" s="20"/>
     </row>
     <row r="12" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="27"/>
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="29"/>
+      <c r="A12" s="31"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="33"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
@@ -1128,16 +1125,16 @@
       <c r="H18" s="10"/>
     </row>
     <row r="19" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="30" t="s">
+      <c r="A19" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="B19" s="31"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="31"/>
-      <c r="G19" s="31"/>
-      <c r="H19" s="32"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="35"/>
+      <c r="F19" s="35"/>
+      <c r="G19" s="35"/>
+      <c r="H19" s="36"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
@@ -1232,14 +1229,14 @@
       <c r="H25" s="10"/>
     </row>
     <row r="26" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="27"/>
-      <c r="B26" s="28"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28"/>
-      <c r="E26" s="28"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="29"/>
+      <c r="A26" s="31"/>
+      <c r="B26" s="32"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="32"/>
+      <c r="G26" s="32"/>
+      <c r="H26" s="33"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
@@ -1390,60 +1387,55 @@
       </c>
       <c r="H36" s="10"/>
     </row>
-    <row r="37" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="23"/>
-      <c r="B37" s="24"/>
-      <c r="C37" s="24"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="24"/>
-      <c r="F37" s="24"/>
-      <c r="G37" s="24"/>
-      <c r="H37" s="25"/>
-    </row>
-    <row r="38" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A38" s="4" t="s">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A37" s="7"/>
+      <c r="B37" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="H37" s="10"/>
+    </row>
+    <row r="38" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="27"/>
+      <c r="B38" s="28"/>
+      <c r="C38" s="28"/>
+      <c r="D38" s="28"/>
+      <c r="E38" s="28"/>
+      <c r="F38" s="28"/>
+      <c r="G38" s="28"/>
+      <c r="H38" s="29"/>
+    </row>
+    <row r="39" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A39" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="B39" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C39" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D38" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="E38" s="6"/>
-      <c r="F38" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G38" s="6"/>
-      <c r="H38" s="19" t="s">
+      <c r="D39" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E39" s="6"/>
+      <c r="F39" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G39" s="6"/>
+      <c r="H39" s="19" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A39" s="11"/>
-      <c r="B39" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="C39" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="F39" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="G39" s="13"/>
-      <c r="H39" s="20"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" s="11"/>
       <c r="B40" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C40" s="12" t="s">
         <v>20</v>
@@ -1459,331 +1451,337 @@
       <c r="H40" s="20"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A41" s="7"/>
-      <c r="B41" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F41" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="H41" s="10"/>
+      <c r="A41" s="11"/>
+      <c r="B41" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D41" s="13"/>
+      <c r="E41" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="F41" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="G41" s="13"/>
+      <c r="H41" s="20"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="7"/>
       <c r="B42" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>6</v>
       </c>
       <c r="H42" s="10"/>
     </row>
-    <row r="43" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="23"/>
-      <c r="B43" s="24"/>
-      <c r="C43" s="24"/>
-      <c r="D43" s="24"/>
-      <c r="E43" s="24"/>
-      <c r="F43" s="24"/>
-      <c r="G43" s="24"/>
-      <c r="H43" s="25"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A44" s="4" t="s">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A43" s="7"/>
+      <c r="B43" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="H43" s="10"/>
+    </row>
+    <row r="44" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="27"/>
+      <c r="B44" s="28"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="28"/>
+      <c r="E44" s="28"/>
+      <c r="F44" s="28"/>
+      <c r="G44" s="28"/>
+      <c r="H44" s="29"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B45" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C44" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="E44" s="6"/>
-      <c r="F44" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G44" s="6"/>
-      <c r="H44" s="19"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A45" s="11"/>
-      <c r="B45" s="12" t="s">
+      <c r="C45" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E45" s="6"/>
+      <c r="F45" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G45" s="6"/>
+      <c r="H45" s="19"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A46" s="11"/>
+      <c r="B46" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="C45" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D45" s="13"/>
-      <c r="E45" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="F45" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="G45" s="13"/>
-      <c r="H45" s="20"/>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A46" s="7"/>
-      <c r="B46" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C46" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F46" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="H46" s="10"/>
+      <c r="C46" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D46" s="13"/>
+      <c r="E46" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="F46" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="G46" s="13"/>
+      <c r="H46" s="20"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="7"/>
       <c r="B47" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F47" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H47" s="10"/>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A48" s="7"/>
+      <c r="B48" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C47" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F47" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="H47" s="10"/>
-    </row>
-    <row r="48" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="23"/>
-      <c r="B48" s="24"/>
-      <c r="C48" s="24"/>
-      <c r="D48" s="24"/>
-      <c r="E48" s="24"/>
-      <c r="F48" s="24"/>
-      <c r="G48" s="24"/>
-      <c r="H48" s="25"/>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A49" s="4" t="s">
+      <c r="C48" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F48" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H48" s="10"/>
+    </row>
+    <row r="49" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="27"/>
+      <c r="B49" s="28"/>
+      <c r="C49" s="28"/>
+      <c r="D49" s="28"/>
+      <c r="E49" s="28"/>
+      <c r="F49" s="28"/>
+      <c r="G49" s="28"/>
+      <c r="H49" s="29"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A50" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B50" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C49" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D49" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="E49" s="6"/>
-      <c r="F49" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G49" s="6"/>
-      <c r="H49" s="19"/>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A50" s="11"/>
-      <c r="B50" s="12" t="s">
+      <c r="C50" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E50" s="6"/>
+      <c r="F50" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="G50" s="6"/>
+      <c r="H50" s="19"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A51" s="11"/>
+      <c r="B51" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="C50" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D50" s="13"/>
-      <c r="E50" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="F50" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="G50" s="13"/>
-      <c r="H50" s="20"/>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A51" s="7"/>
-      <c r="B51" s="8" t="s">
+      <c r="C51" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D51" s="13"/>
+      <c r="E51" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="F51" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="G51" s="13"/>
+      <c r="H51" s="20"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A52" s="7"/>
+      <c r="B52" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C51" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F51" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="H51" s="10"/>
-    </row>
-    <row r="52" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="16"/>
-      <c r="B52" s="17"/>
-      <c r="C52" s="17"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="14"/>
-      <c r="F52" s="14"/>
-      <c r="G52" s="14"/>
-      <c r="H52" s="21"/>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A53" s="4" t="s">
+      <c r="C52" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H52" s="10"/>
+    </row>
+    <row r="53" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="16"/>
+      <c r="B53" s="17"/>
+      <c r="C53" s="17"/>
+      <c r="D53" s="14"/>
+      <c r="E53" s="14"/>
+      <c r="F53" s="14"/>
+      <c r="G53" s="14"/>
+      <c r="H53" s="21"/>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A54" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B53" s="5" t="s">
+      <c r="B54" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C53" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D53" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="E53" s="6"/>
-      <c r="F53" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G53" s="6"/>
-      <c r="H53" s="19"/>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A54" s="7"/>
-      <c r="B54" s="8" t="s">
+      <c r="C54" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E54" s="6"/>
+      <c r="F54" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G54" s="6"/>
+      <c r="H54" s="19"/>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A55" s="7"/>
+      <c r="B55" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C54" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F54" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="H54" s="10"/>
-    </row>
-    <row r="55" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="23"/>
-      <c r="B55" s="24"/>
-      <c r="C55" s="24"/>
-      <c r="D55" s="24"/>
-      <c r="E55" s="24"/>
-      <c r="F55" s="24"/>
-      <c r="G55" s="24"/>
-      <c r="H55" s="25"/>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A56" s="33" t="s">
+      <c r="C55" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F55" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H55" s="10"/>
+    </row>
+    <row r="56" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="27"/>
+      <c r="B56" s="28"/>
+      <c r="C56" s="28"/>
+      <c r="D56" s="28"/>
+      <c r="E56" s="28"/>
+      <c r="F56" s="28"/>
+      <c r="G56" s="28"/>
+      <c r="H56" s="29"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A57" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="B56" s="34" t="s">
+      <c r="B57" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="C56" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="D56" s="35" t="s">
-        <v>37</v>
-      </c>
-      <c r="E56" s="35"/>
-      <c r="F56" s="35" t="s">
-        <v>7</v>
-      </c>
-      <c r="G56" s="35"/>
-      <c r="H56" s="36"/>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A57" s="7"/>
-      <c r="B57" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="C57" s="37" t="s">
-        <v>20</v>
-      </c>
-      <c r="D57" s="38"/>
-      <c r="E57" s="38" t="s">
-        <v>37</v>
-      </c>
-      <c r="F57" s="38" t="s">
-        <v>7</v>
-      </c>
-      <c r="G57" s="38"/>
-      <c r="H57" s="10"/>
+      <c r="C57" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="D57" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="E57" s="25"/>
+      <c r="F57" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="G57" s="25"/>
+      <c r="H57" s="26"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="7"/>
-      <c r="B58" s="37" t="s">
-        <v>25</v>
-      </c>
-      <c r="C58" s="37" t="s">
-        <v>18</v>
-      </c>
-      <c r="D58" s="38"/>
-      <c r="E58" s="38"/>
-      <c r="F58" s="38" t="s">
-        <v>7</v>
-      </c>
-      <c r="G58" s="38"/>
-      <c r="H58" s="10" t="s">
-        <v>66</v>
-      </c>
+      <c r="B58" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E58" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F58" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H58" s="10"/>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="7"/>
-      <c r="B59" s="37" t="s">
-        <v>62</v>
-      </c>
-      <c r="C59" s="37" t="s">
-        <v>18</v>
-      </c>
-      <c r="D59" s="38"/>
-      <c r="E59" s="38"/>
-      <c r="F59" s="38" t="s">
-        <v>7</v>
-      </c>
-      <c r="G59" s="38"/>
+      <c r="B59" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F59" s="9" t="s">
+        <v>7</v>
+      </c>
       <c r="H59" s="10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="7"/>
-      <c r="B60" s="37" t="s">
+      <c r="B60" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F60" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H60" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A61" s="7"/>
+      <c r="B61" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C60" s="37" t="s">
-        <v>20</v>
-      </c>
-      <c r="D60" s="38"/>
-      <c r="E60" s="38"/>
-      <c r="F60" s="38"/>
-      <c r="G60" s="38"/>
-      <c r="H60" s="10"/>
-    </row>
-    <row r="61" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="16"/>
-      <c r="B61" s="17" t="s">
+      <c r="C61" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H61" s="10"/>
+    </row>
+    <row r="62" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A62" s="16"/>
+      <c r="B62" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="C61" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="D61" s="14"/>
-      <c r="E61" s="14"/>
-      <c r="F61" s="14"/>
-      <c r="G61" s="14"/>
-      <c r="H61" s="21"/>
+      <c r="C62" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="D62" s="14"/>
+      <c r="E62" s="14"/>
+      <c r="F62" s="14"/>
+      <c r="G62" s="14"/>
+      <c r="H62" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A55:H55"/>
+    <mergeCell ref="A49:H49"/>
+    <mergeCell ref="A56:H56"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A19:H19"/>
     <mergeCell ref="A26:H26"/>
-    <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A44:H44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(db): discard agent_execution "CANCELLED" state
</commit_message>
<xml_diff>
--- a/database/data_dictionary.xlsx
+++ b/database/data_dictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Duck\Desktop\Taller\veraud\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8BBD8D1-9063-44C9-B9B6-F60DC68F3822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{561BAF3E-1373-4DB4-8E95-BC14B8472BE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{C4133E00-A44A-4AC3-8FAA-A9370F47246C}"/>
   </bookViews>
@@ -206,9 +206,6 @@
     <t>Values: "QUEUED", "RUNNING", "COMPLETED", "FAILED", "CANCELLED"</t>
   </si>
   <si>
-    <t>Values: "QUEUED", "ANALYZING", "COMPLETED", "FAILED", "CANCELLED"</t>
-  </si>
-  <si>
     <t>Values:  "QUEUED", "READY", "SYNCING"</t>
   </si>
   <si>
@@ -240,6 +237,9 @@
   </si>
   <si>
     <t>result</t>
+  </si>
+  <si>
+    <t>Values: "WAITING", "RUNNING", "COMPLETED", "FAILED"</t>
   </si>
 </sst>
 </file>
@@ -959,7 +959,7 @@
         <v>7</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
@@ -1108,7 +1108,7 @@
         <v>7</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
@@ -1126,7 +1126,7 @@
     </row>
     <row r="19" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="34" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B19" s="35"/>
       <c r="C19" s="35"/>
@@ -1186,7 +1186,7 @@
         <v>7</v>
       </c>
       <c r="H22" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
@@ -1390,7 +1390,7 @@
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="7"/>
       <c r="B37" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>18</v>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G39" s="6"/>
       <c r="H39" s="19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
@@ -1684,7 +1684,7 @@
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B57" s="24" t="s">
         <v>5</v>
@@ -1730,13 +1730,13 @@
         <v>7</v>
       </c>
       <c r="H59" s="10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="7"/>
       <c r="B60" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C60" s="8" t="s">
         <v>18</v>
@@ -1745,13 +1745,13 @@
         <v>7</v>
       </c>
       <c r="H60" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="7"/>
       <c r="B61" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C61" s="8" t="s">
         <v>20</v>
@@ -1761,7 +1761,7 @@
     <row r="62" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A62" s="16"/>
       <c r="B62" s="17" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C62" s="17" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
docs(database): mark evaluation_id nullable
</commit_message>
<xml_diff>
--- a/database/data_dictionary.xlsx
+++ b/database/data_dictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Duck\Desktop\Taller\veraud\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{561BAF3E-1373-4DB4-8E95-BC14B8472BE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4317891B-5659-42E5-BB88-880B0277B615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{C4133E00-A44A-4AC3-8FAA-A9370F47246C}"/>
   </bookViews>
@@ -1271,7 +1271,7 @@
         <v>37</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G28" s="13"/>
       <c r="H28" s="20"/>

</xml_diff>